<commit_message>
Fix for YSI700 resistance/temp equation.
Updated the algorithm to contain the equation that, during testing, responds correctly
on the patient monitors. I'm not sure why the original table isn't working. But, after
testing the values in the new equation on two separate ECGs, this equation works.
</commit_message>
<xml_diff>
--- a/YSI700.xlsx
+++ b/YSI700.xlsx
@@ -203,10 +203,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.168266117162202"/>
-          <c:y val="0.0396834984295724"/>
-          <c:w val="0.799941124521637"/>
-          <c:h val="0.693404203913989"/>
+          <c:x val="0.168273753527752"/>
+          <c:y val="0.039685895499849"/>
+          <c:w val="0.79991768579492"/>
+          <c:h val="0.693385684083359"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -355,11 +355,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="81448917"/>
-        <c:axId val="83086586"/>
+        <c:axId val="67103285"/>
+        <c:axId val="1823398"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="81448917"/>
+        <c:axId val="67103285"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -424,12 +424,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83086586"/>
+        <c:crossAx val="1823398"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="83086586"/>
+        <c:axId val="1823398"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -494,7 +494,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81448917"/>
+        <c:crossAx val="67103285"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -535,9 +535,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>782280</xdr:colOff>
+      <xdr:colOff>781920</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>47160</xdr:rowOff>
+      <xdr:rowOff>46800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -545,8 +545,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="2006280" y="102240"/>
-        <a:ext cx="6114240" cy="5959800"/>
+        <a:off x="2008800" y="102240"/>
+        <a:ext cx="6122520" cy="5959440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -565,7 +565,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
2.1-alpha.1 - complete rewrite
Now factors in dividing resistors to increase range accuracy

Can now calculate and draw both YSI400 and 700 ranges on the same graph.

Includes calibration steps.
</commit_message>
<xml_diff>
--- a/YSI700.xlsx
+++ b/YSI700.xlsx
@@ -136,7 +136,7 @@
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFF1493"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
@@ -191,7 +191,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -203,10 +203,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.168273753527752"/>
-          <c:y val="0.039685895499849"/>
-          <c:w val="0.79991768579492"/>
-          <c:h val="0.693385684083359"/>
+          <c:x val="0.168271488961954"/>
+          <c:y val="0.0396882928597318"/>
+          <c:w val="0.799847346171912"/>
+          <c:h val="0.693367162015223"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -217,11 +217,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$B$1</c:f>
+              <c:f>Sheet1!$B$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Resistance</c:v>
+                  <c:v>6270</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -270,7 +270,7 @@
             <c:spPr>
               <a:ln w="0">
                 <a:solidFill>
-                  <a:srgbClr val="004586"/>
+                  <a:srgbClr val="ff1493"/>
                 </a:solidFill>
               </a:ln>
             </c:spPr>
@@ -283,35 +283,56 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$10</c:f>
+              <c:f>Sheet1!$A$3:$A$18</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>25</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>30</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="7">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>35</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="11">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="15">
                   <c:v>40</c:v>
                 </c:pt>
               </c:numCache>
@@ -319,47 +340,68 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$10</c:f>
+              <c:f>Sheet1!$B$3:$B$18</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="9"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
-                  <c:v>94980</c:v>
+                  <c:v>6000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>74445</c:v>
+                  <c:v>5744</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>58748</c:v>
+                  <c:v>5500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46666</c:v>
+                  <c:v>5266</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>37303</c:v>
+                  <c:v>5046</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30000</c:v>
+                  <c:v>4834</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>24268</c:v>
+                  <c:v>4634</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>19741</c:v>
+                  <c:v>4442</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16146</c:v>
+                  <c:v>4260</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4084</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3918</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3760</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3610</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3466</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3328</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3196</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="67103285"/>
-        <c:axId val="1823398"/>
+        <c:axId val="82845653"/>
+        <c:axId val="45336748"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="67103285"/>
+        <c:axId val="82845653"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -424,14 +466,16 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1823398"/>
+        <c:crossAx val="45336748"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1823398"/>
+        <c:axId val="45336748"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="6500"/>
+          <c:min val="3000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -494,8 +538,8 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67103285"/>
-        <c:crosses val="autoZero"/>
+        <c:crossAx val="82845653"/>
+        <c:crossesAt val="0"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
@@ -535,9 +579,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>781920</xdr:colOff>
+      <xdr:colOff>781560</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>46800</xdr:rowOff>
+      <xdr:rowOff>46440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -545,8 +589,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="2008800" y="102240"/>
-        <a:ext cx="6122520" cy="5959440"/>
+        <a:off x="2011320" y="102240"/>
+        <a:ext cx="6131160" cy="5959080"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -564,8 +608,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -577,50 +621,50 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>94980</v>
+        <v>6270</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>74445</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>58748</v>
+        <v>5744</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46666</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>37303</v>
+        <v>5266</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>30000</v>
+        <v>5046</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -628,23 +672,87 @@
         <v>30</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>24268</v>
+        <v>4834</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>19741</v>
+        <v>4634</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>4442</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>4260</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>4084</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>3918</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>3760</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>3610</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>3466</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>3328</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="B10" s="1" t="n">
-        <v>16146</v>
+      <c r="B18" s="0" t="n">
+        <v>3196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>